<commit_message>
Detaille les frais de notaire en taxes gouvernementales et honoraires
Remplace la ligne unique a 6% par deux lignes parametrees : 5% de taxes
gouvernementales et 1% d'honoraires du notaire, avec un sous-total notaire.
Les totaux et l'acompte restent inchanges.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014vwehdk7pAYrgh8aPNjCvp
</commit_message>
<xml_diff>
--- a/transactions/Recap_transaction_fonciere_appel_de_fonds.xlsx
+++ b/transactions/Recap_transaction_fonciere_appel_de_fonds.xlsx
@@ -156,7 +156,12 @@
     </comment>
     <comment ref="B13" authorId="0" shapeId="0">
       <text>
-        <t>Frais de notaire calcules sur le prix client (prix avec commission). Hypothese : 6% indique par l'agent.</t>
+        <t>Taxes gouvernementales : 5% du prix client (prix avec commission). Hypothese indiquee par l'agent.</t>
+      </text>
+    </comment>
+    <comment ref="B14" authorId="0" shapeId="0">
+      <text>
+        <t>Honoraires du notaire : 1% du prix client (prix avec commission). Hypothese indiquee par l'agent.</t>
       </text>
     </comment>
   </commentList>
@@ -452,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -562,103 +567,86 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Taux frais de notaire</t>
+          <t>Taxes gouvernementales (% du prix client)</t>
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Frais de geometre (EUR)</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="n">
-        <v>1000</v>
+          <t>Honoraires du notaire (% du prix client)</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0.01</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
+          <t>Frais de geometre (EUR)</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
           <t>Taux d'acompte (appel de fonds)</t>
         </is>
       </c>
-      <c r="B15" s="5" t="n">
+      <c r="B16" s="5" t="n">
         <v>0.1</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>DETAIL DU CALCUL</t>
-        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
+          <t>DETAIL DU CALCUL</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
           <t>Poste</t>
         </is>
       </c>
-      <c r="B18" s="1" t="inlineStr">
+      <c r="B19" s="1" t="inlineStr">
         <is>
           <t>Surface (ares)</t>
         </is>
       </c>
-      <c r="C18" s="1" t="inlineStr">
+      <c r="C19" s="1" t="inlineStr">
         <is>
           <t>Duree (ans)</t>
         </is>
       </c>
-      <c r="D18" s="1" t="inlineStr">
+      <c r="D19" s="1" t="inlineStr">
         <is>
           <t>Prix unitaire (IDR/are/an)</t>
         </is>
       </c>
-      <c r="E18" s="1" t="inlineStr">
+      <c r="E19" s="1" t="inlineStr">
         <is>
           <t>Montant IDR</t>
         </is>
       </c>
-      <c r="F18" s="1" t="inlineStr">
+      <c r="F19" s="1" t="inlineStr">
         <is>
           <t>Montant EUR</t>
         </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Prix du terrain - PRIX VENDEUR</t>
-        </is>
-      </c>
-      <c r="B19" s="3">
-        <f>B7</f>
-        <v/>
-      </c>
-      <c r="C19" s="4">
-        <f>B9</f>
-        <v/>
-      </c>
-      <c r="D19" s="4">
-        <f>B10</f>
-        <v/>
-      </c>
-      <c r="E19" s="4">
-        <f>B19*C19*D19</f>
-        <v/>
-      </c>
-      <c r="F19" s="3">
-        <f>E19/$B$12</f>
-        <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Prix du terrain - PRIX CLIENT (avec commission)</t>
+          <t>Prix du terrain - PRIX VENDEUR</t>
         </is>
       </c>
       <c r="B20" s="3">
@@ -670,7 +658,7 @@
         <v/>
       </c>
       <c r="D20" s="4">
-        <f>B11</f>
+        <f>B10</f>
         <v/>
       </c>
       <c r="E20" s="4">
@@ -685,11 +673,23 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>dont commission agence (ecart vendeur / client)</t>
-        </is>
+          <t>Prix du terrain - PRIX CLIENT (avec commission)</t>
+        </is>
+      </c>
+      <c r="B21" s="3">
+        <f>B7</f>
+        <v/>
+      </c>
+      <c r="C21" s="4">
+        <f>B9</f>
+        <v/>
+      </c>
+      <c r="D21" s="4">
+        <f>B11</f>
+        <v/>
       </c>
       <c r="E21" s="4">
-        <f>E20-E19</f>
+        <f>B21*C21*D21</f>
         <v/>
       </c>
       <c r="F21" s="3">
@@ -697,81 +697,108 @@
         <v/>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="1" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>dont commission agence (ecart vendeur / client)</t>
+        </is>
+      </c>
+      <c r="E22" s="4">
+        <f>E21-E20</f>
+        <v/>
+      </c>
+      <c r="F22" s="3">
+        <f>E22/$B$12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
         <is>
           <t>FRAIS ANNEXES</t>
         </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Frais de notaire (6% du prix client)</t>
-        </is>
-      </c>
-      <c r="D24" s="5">
-        <f>B13</f>
-        <v/>
-      </c>
-      <c r="E24" s="4">
-        <f>E20*$B$13</f>
-        <v/>
-      </c>
-      <c r="F24" s="3">
-        <f>E24/$B$12</f>
-        <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
+          <t>Taxes gouvernementales (5% du prix client)</t>
+        </is>
+      </c>
+      <c r="D25" s="5">
+        <f>B13</f>
+        <v/>
+      </c>
+      <c r="E25" s="4">
+        <f>E21*$B$13</f>
+        <v/>
+      </c>
+      <c r="F25" s="3">
+        <f>E25/$B$12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Honoraires du notaire (1% du prix client)</t>
+        </is>
+      </c>
+      <c r="D26" s="5">
+        <f>B14</f>
+        <v/>
+      </c>
+      <c r="E26" s="4">
+        <f>E21*$B$14</f>
+        <v/>
+      </c>
+      <c r="F26" s="3">
+        <f>E26/$B$12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Sous-total frais de notaire (taxes + honoraires)</t>
+        </is>
+      </c>
+      <c r="D27" s="5">
+        <f>B13+B14</f>
+        <v/>
+      </c>
+      <c r="E27" s="4">
+        <f>E25+E26</f>
+        <v/>
+      </c>
+      <c r="F27" s="3">
+        <f>E27/$B$12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
           <t>Frais de geometre (forfait 1 000 EUR)</t>
         </is>
       </c>
-      <c r="E25" s="4">
-        <f>$B$14*$B$12</f>
-        <v/>
-      </c>
-      <c r="F25" s="3">
-        <f>$B$14</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="1" t="inlineStr">
+      <c r="E28" s="4">
+        <f>$B$15*$B$12</f>
+        <v/>
+      </c>
+      <c r="F28" s="3">
+        <f>$B$15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="inlineStr">
         <is>
           <t>TOTAL DE L'OPERATION POUR L'ACHETEUR</t>
         </is>
       </c>
-      <c r="E27" s="6">
-        <f>E20+E24+E25</f>
-        <v/>
-      </c>
-      <c r="F27" s="7">
-        <f>E27/$B$12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="1" t="inlineStr">
-        <is>
-          <t>APPEL DE FONDS</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>Acompte 10% du total de l'operation (reservation notaire)</t>
-        </is>
-      </c>
-      <c r="D30" s="5">
-        <f>B15</f>
-        <v/>
-      </c>
       <c r="E30" s="6">
-        <f>E27*$B$15</f>
+        <f>E21+E27+E28</f>
         <v/>
       </c>
       <c r="F30" s="7">
@@ -779,75 +806,108 @@
         <v/>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>Solde a regler apres acompte</t>
-        </is>
-      </c>
-      <c r="E31" s="4">
-        <f>E27-E30</f>
-        <v/>
-      </c>
-      <c r="F31" s="3">
-        <f>E31/$B$12</f>
-        <v/>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>APPEL DE FONDS</t>
+        </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Pour information : 10% du prix du terrain seul</t>
-        </is>
-      </c>
-      <c r="E33" s="4">
-        <f>E20*$B$15</f>
-        <v/>
-      </c>
-      <c r="F33" s="3">
+          <t>Acompte 10% du total de l'operation (reservation notaire)</t>
+        </is>
+      </c>
+      <c r="D33" s="5">
+        <f>B16</f>
+        <v/>
+      </c>
+      <c r="E33" s="6">
+        <f>E30*$B$16</f>
+        <v/>
+      </c>
+      <c r="F33" s="7">
         <f>E33/$B$12</f>
         <v/>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="1" t="inlineStr">
-        <is>
-          <t>NOTES / HYPOTHESES</t>
-        </is>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Solde a regler apres acompte</t>
+        </is>
+      </c>
+      <c r="E34" s="4">
+        <f>E30-E33</f>
+        <v/>
+      </c>
+      <c r="F34" s="3">
+        <f>E34/$B$12</f>
+        <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>1 are = 100 m2 -&gt; terrain de 600 m2. Prix leasehold exprime en IDR par are et par an, sur 30 ans.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>Taux de change en B12 : reference BCE du 20/08/2026 (1 EUR = 20 788,62 IDR). A actualiser avant envoi au client.</t>
-        </is>
+          <t>Pour information : 10% du prix du terrain seul</t>
+        </is>
+      </c>
+      <c r="E36" s="4">
+        <f>E21*$B$16</f>
+        <v/>
+      </c>
+      <c r="F36" s="3">
+        <f>E36/$B$12</f>
+        <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>Frais de notaire (B13) calcules sur le prix client avec commission. Modifier la formule en E24 si la base retenue est le prix vendeur.</t>
+      <c r="A38" s="1" t="inlineStr">
+        <is>
+          <t>NOTES / HYPOTHESES</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Frais de geometre saisis en EUR (B14) et convertis en IDR au taux B12.</t>
+          <t>1 are = 100 m2 -&gt; terrain de 600 m2. Prix leasehold exprime en IDR par are et par an, sur 30 ans.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Seules les cellules de parametres (colonne B, lignes 7 a 15) sont a saisir : tout le reste du tableau est calcule par formules et se met a jour automatiquement.</t>
+          <t>Taux de change en B12 : reference BCE du 20/08/2026 (1 EUR = 20 788,62 IDR). A actualiser avant envoi au client.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Frais de notaire detailles : 5% de taxes gouvernementales (B13) + 1% d'honoraires du notaire (B14), soit 6% au total.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Ces deux taux sont appliques au prix client avec commission. Remplacer E21 par E20 dans les formules E25 et E26 si la base retenue est le prix vendeur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Frais de geometre saisis en EUR (B15) et convertis en IDR au taux B12.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Seules les cellules de parametres (colonne B, lignes 7 a 16) sont a saisir : tout le reste du tableau est calcule par formules et se met a jour automatiquement.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Applique un forfait plancher de 10 000 000 IDR aux honoraires du notaire
Les honoraires prennent desormais le maximum entre 1% du prix client et un
forfait minimum parametrable (B15, 10 000 000 IDR). La colonne des taux
affiche le taux reellement supporte.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014vwehdk7pAYrgh8aPNjCvp
</commit_message>
<xml_diff>
--- a/transactions/Recap_transaction_fonciere_appel_de_fonds.xlsx
+++ b/transactions/Recap_transaction_fonciere_appel_de_fonds.xlsx
@@ -164,6 +164,17 @@
         <t>Honoraires du notaire : 1% du prix client (prix avec commission). Hypothese indiquee par l'agent.</t>
       </text>
     </comment>
+    <comment ref="B15" authorId="0" shapeId="0">
+      <text>
+        <t>Forfait plancher : si 1% du prix client donne moins de 10 000 000 IDR, ce forfait s'applique a la place du pourcentage.</t>
+      </text>
+    </comment>
+    <comment ref="E27" authorId="0" shapeId="0">
+      <text>
+        <t>MAX entre 1% du prix client et le forfait minimum de la cellule B15 : si le pourcentage donne moins de 10 000 000 IDR, c'est le forfait qui s'applique.
+La colonne D affiche le taux reellement supporte.</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -457,10 +468,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
@@ -587,93 +598,76 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Frais de geometre (EUR)</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="n">
-        <v>1000</v>
+          <t>Honoraires du notaire - forfait minimum (IDR)</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>10000000</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>Frais de geometre (EUR)</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
           <t>Taux d'acompte (appel de fonds)</t>
         </is>
       </c>
-      <c r="B16" s="5" t="n">
+      <c r="B17" s="5" t="n">
         <v>0.1</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>DETAIL DU CALCUL</t>
-        </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
+          <t>DETAIL DU CALCUL</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
           <t>Poste</t>
         </is>
       </c>
-      <c r="B19" s="1" t="inlineStr">
+      <c r="B20" s="1" t="inlineStr">
         <is>
           <t>Surface (ares)</t>
         </is>
       </c>
-      <c r="C19" s="1" t="inlineStr">
+      <c r="C20" s="1" t="inlineStr">
         <is>
           <t>Duree (ans)</t>
         </is>
       </c>
-      <c r="D19" s="1" t="inlineStr">
+      <c r="D20" s="1" t="inlineStr">
         <is>
           <t>Prix unitaire (IDR/are/an)</t>
         </is>
       </c>
-      <c r="E19" s="1" t="inlineStr">
+      <c r="E20" s="1" t="inlineStr">
         <is>
           <t>Montant IDR</t>
         </is>
       </c>
-      <c r="F19" s="1" t="inlineStr">
+      <c r="F20" s="1" t="inlineStr">
         <is>
           <t>Montant EUR</t>
         </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Prix du terrain - PRIX VENDEUR</t>
-        </is>
-      </c>
-      <c r="B20" s="3">
-        <f>B7</f>
-        <v/>
-      </c>
-      <c r="C20" s="4">
-        <f>B9</f>
-        <v/>
-      </c>
-      <c r="D20" s="4">
-        <f>B10</f>
-        <v/>
-      </c>
-      <c r="E20" s="4">
-        <f>B20*C20*D20</f>
-        <v/>
-      </c>
-      <c r="F20" s="3">
-        <f>E20/$B$12</f>
-        <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Prix du terrain - PRIX CLIENT (avec commission)</t>
+          <t>Prix du terrain - PRIX VENDEUR</t>
         </is>
       </c>
       <c r="B21" s="3">
@@ -685,7 +679,7 @@
         <v/>
       </c>
       <c r="D21" s="4">
-        <f>B11</f>
+        <f>B10</f>
         <v/>
       </c>
       <c r="E21" s="4">
@@ -700,11 +694,23 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>dont commission agence (ecart vendeur / client)</t>
-        </is>
+          <t>Prix du terrain - PRIX CLIENT (avec commission)</t>
+        </is>
+      </c>
+      <c r="B22" s="3">
+        <f>B7</f>
+        <v/>
+      </c>
+      <c r="C22" s="4">
+        <f>B9</f>
+        <v/>
+      </c>
+      <c r="D22" s="4">
+        <f>B11</f>
+        <v/>
       </c>
       <c r="E22" s="4">
-        <f>E21-E20</f>
+        <f>B22*C22*D22</f>
         <v/>
       </c>
       <c r="F22" s="3">
@@ -712,44 +718,40 @@
         <v/>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="1" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>dont commission agence (ecart vendeur / client)</t>
+        </is>
+      </c>
+      <c r="E23" s="4">
+        <f>E22-E21</f>
+        <v/>
+      </c>
+      <c r="F23" s="3">
+        <f>E23/$B$12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
         <is>
           <t>FRAIS ANNEXES</t>
         </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Taxes gouvernementales (5% du prix client)</t>
-        </is>
-      </c>
-      <c r="D25" s="5">
-        <f>B13</f>
-        <v/>
-      </c>
-      <c r="E25" s="4">
-        <f>E21*$B$13</f>
-        <v/>
-      </c>
-      <c r="F25" s="3">
-        <f>E25/$B$12</f>
-        <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Honoraires du notaire (1% du prix client)</t>
+          <t>Taxes gouvernementales (5% du prix client)</t>
         </is>
       </c>
       <c r="D26" s="5">
-        <f>B14</f>
+        <f>B13</f>
         <v/>
       </c>
       <c r="E26" s="4">
-        <f>E21*$B$14</f>
+        <f>E22*$B$13</f>
         <v/>
       </c>
       <c r="F26" s="3">
@@ -760,15 +762,15 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Sous-total frais de notaire (taxes + honoraires)</t>
+          <t>Honoraires du notaire (1% du prix client, minimum 10 000 000 IDR)</t>
         </is>
       </c>
       <c r="D27" s="5">
-        <f>B13+B14</f>
+        <f>IF(E22=0,0,E27/E22)</f>
         <v/>
       </c>
       <c r="E27" s="4">
-        <f>E25+E26</f>
+        <f>MAX(E22*$B$14,$B$15)</f>
         <v/>
       </c>
       <c r="F27" s="3">
@@ -779,135 +781,161 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t>Sous-total frais de notaire (taxes + honoraires)</t>
+        </is>
+      </c>
+      <c r="D28" s="5">
+        <f>IF(E22=0,0,E28/E22)</f>
+        <v/>
+      </c>
+      <c r="E28" s="4">
+        <f>E26+E27</f>
+        <v/>
+      </c>
+      <c r="F28" s="3">
+        <f>E28/$B$12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
           <t>Frais de geometre (forfait 1 000 EUR)</t>
         </is>
       </c>
-      <c r="E28" s="4">
-        <f>$B$15*$B$12</f>
-        <v/>
-      </c>
-      <c r="F28" s="3">
-        <f>$B$15</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="1" t="inlineStr">
+      <c r="E29" s="4">
+        <f>$B$16*$B$12</f>
+        <v/>
+      </c>
+      <c r="F29" s="3">
+        <f>$B$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr">
         <is>
           <t>TOTAL DE L'OPERATION POUR L'ACHETEUR</t>
         </is>
       </c>
-      <c r="E30" s="6">
-        <f>E21+E27+E28</f>
-        <v/>
-      </c>
-      <c r="F30" s="7">
-        <f>E30/$B$12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="1" t="inlineStr">
+      <c r="E31" s="6">
+        <f>E22+E28+E29</f>
+        <v/>
+      </c>
+      <c r="F31" s="7">
+        <f>E31/$B$12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="inlineStr">
         <is>
           <t>APPEL DE FONDS</t>
         </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>Acompte 10% du total de l'operation (reservation notaire)</t>
-        </is>
-      </c>
-      <c r="D33" s="5">
-        <f>B16</f>
-        <v/>
-      </c>
-      <c r="E33" s="6">
-        <f>E30*$B$16</f>
-        <v/>
-      </c>
-      <c r="F33" s="7">
-        <f>E33/$B$12</f>
-        <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
+          <t>Acompte 10% du total de l'operation (reservation notaire)</t>
+        </is>
+      </c>
+      <c r="D34" s="5">
+        <f>B17</f>
+        <v/>
+      </c>
+      <c r="E34" s="6">
+        <f>E31*$B$17</f>
+        <v/>
+      </c>
+      <c r="F34" s="7">
+        <f>E34/$B$12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
           <t>Solde a regler apres acompte</t>
         </is>
       </c>
-      <c r="E34" s="4">
-        <f>E30-E33</f>
-        <v/>
-      </c>
-      <c r="F34" s="3">
-        <f>E34/$B$12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="E35" s="4">
+        <f>E31-E34</f>
+        <v/>
+      </c>
+      <c r="F35" s="3">
+        <f>E35/$B$12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>Pour information : 10% du prix du terrain seul</t>
         </is>
       </c>
-      <c r="E36" s="4">
-        <f>E21*$B$16</f>
-        <v/>
-      </c>
-      <c r="F36" s="3">
-        <f>E36/$B$12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="1" t="inlineStr">
+      <c r="E37" s="4">
+        <f>E22*$B$17</f>
+        <v/>
+      </c>
+      <c r="F37" s="3">
+        <f>E37/$B$12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="inlineStr">
         <is>
           <t>NOTES / HYPOTHESES</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>1 are = 100 m2 -&gt; terrain de 600 m2. Prix leasehold exprime en IDR par are et par an, sur 30 ans.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Taux de change en B12 : reference BCE du 20/08/2026 (1 EUR = 20 788,62 IDR). A actualiser avant envoi au client.</t>
+          <t>1 are = 100 m2 -&gt; terrain de 600 m2. Prix leasehold exprime en IDR par are et par an, sur 30 ans.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Frais de notaire detailles : 5% de taxes gouvernementales (B13) + 1% d'honoraires du notaire (B14), soit 6% au total.</t>
+          <t>Taux de change en B12 : reference BCE du 20/08/2026 (1 EUR = 20 788,62 IDR). A actualiser avant envoi au client.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Ces deux taux sont appliques au prix client avec commission. Remplacer E21 par E20 dans les formules E25 et E26 si la base retenue est le prix vendeur.</t>
+          <t>Frais de notaire detailles : taxes gouvernementales 5% (B13) + honoraires du notaire 1% (B14).</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Frais de geometre saisis en EUR (B15) et convertis en IDR au taux B12.</t>
+          <t>Honoraires du notaire : le pourcentage s'applique sauf s'il donne moins que le forfait minimum de 10 000 000 IDR (B15), auquel cas le forfait est retenu (formule MAX en E27).</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Seules les cellules de parametres (colonne B, lignes 7 a 16) sont a saisir : tout le reste du tableau est calcule par formules et se met a jour automatiquement.</t>
+          <t>Ces taux sont appliques au prix client avec commission. Remplacer E22 par E21 dans les formules E26 et E27 si la base retenue est le prix vendeur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Frais de geometre saisis en EUR (B16) et convertis en IDR au taux B12.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Seules les cellules de parametres (colonne B, lignes 7 a 17) sont a saisir : tout le reste du tableau est calcule par formules et se met a jour automatiquement.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajoute la version freehold du recapitulatif et factorise le generateur
Le generateur produit desormais les deux tableaux depuis une source unique :
la version leasehold (prix par are et par an x duree) et la version freehold
(prix par are, sans duree). Frais de notaire, geometre, total et acompte sont
identiques dans les deux cas. Une ligne 'Regime' identifie chaque tableau.
Les deux prix au are du tableau freehold sont laisses a saisir.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014vwehdk7pAYrgh8aPNjCvp
</commit_message>
<xml_diff>
--- a/transactions/Recap_transaction_fonciere_appel_de_fonds.xlsx
+++ b/transactions/Recap_transaction_fonciere_appel_de_fonds.xlsx
@@ -148,31 +148,31 @@
     <author>Agence</author>
   </authors>
   <commentList>
-    <comment ref="B12" authorId="0" shapeId="0">
+    <comment ref="B13" authorId="0" shapeId="0">
       <text>
         <t>Taux de reference BCE du 20/08/2026 : 1 EUR = 20 788,62 IDR (source : api.frankfurter.dev).
 A actualiser au taux du jour / au taux retenu avec le client.</t>
       </text>
     </comment>
-    <comment ref="B13" authorId="0" shapeId="0">
+    <comment ref="B14" authorId="0" shapeId="0">
       <text>
         <t>Taxes gouvernementales : 5% du prix client (prix avec commission). Hypothese indiquee par l'agent.</t>
       </text>
     </comment>
-    <comment ref="B14" authorId="0" shapeId="0">
+    <comment ref="B15" authorId="0" shapeId="0">
       <text>
         <t>Honoraires du notaire : 1% du prix client (prix avec commission). Hypothese indiquee par l'agent.</t>
       </text>
     </comment>
-    <comment ref="B15" authorId="0" shapeId="0">
+    <comment ref="B16" authorId="0" shapeId="0">
       <text>
-        <t>Forfait plancher : si 1% du prix client donne moins de 10 000 000 IDR, ce forfait s'applique a la place du pourcentage.</t>
+        <t>Forfait plancher : si le pourcentage donne moins de 10 000 000 IDR, ce forfait s'applique a la place du pourcentage.</t>
       </text>
     </comment>
-    <comment ref="E27" authorId="0" shapeId="0">
+    <comment ref="E28" authorId="0" shapeId="0">
       <text>
-        <t>MAX entre 1% du prix client et le forfait minimum de la cellule B15 : si le pourcentage donne moins de 10 000 000 IDR, c'est le forfait qui s'applique.
-La colonne D affiche le taux reellement supporte.</t>
+        <t>MAX entre le pourcentage d'honoraires et le forfait minimum : si le pourcentage donne moins de 10 000 000 IDR, c'est le forfait qui s'applique.
+La colonne des taux affiche le taux reellement supporte.</t>
       </text>
     </comment>
   </commentList>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -487,226 +487,206 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Client :</t>
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Regime : LEASEHOLD (bail 30 ans)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Terrain / localisation :</t>
+          <t>Client :</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t>Terrain / localisation :</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
           <t>Date :</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>PARAMETRES (cellules a modifier)</t>
         </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Surface du terrain (ares)</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Surface du terrain (m2)</t>
-        </is>
-      </c>
-      <c r="B8" s="4">
-        <f>B7*100</f>
-        <v/>
+          <t>Surface du terrain (ares)</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Duree du leasehold (annees)</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="n">
-        <v>30</v>
+          <t>Surface du terrain (m2)</t>
+        </is>
+      </c>
+      <c r="B9" s="4">
+        <f>B8*100</f>
+        <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Prix vendeur (IDR / are / an)</t>
+          <t>Duree du leasehold (annees)</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>4000000</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Prix client avec commission (IDR / are / an)</t>
+          <t>Prix vendeur (IDR / are / an)</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>5000000</v>
+        <v>4000000</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Taux de change (IDR pour 1 EUR)</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="n">
-        <v>20788.62</v>
+          <t>Prix client avec commission (IDR / are / an)</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>5000000</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Taxes gouvernementales (% du prix client)</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="n">
-        <v>0.05</v>
+          <t>Taux de change (IDR pour 1 EUR)</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>20788.62</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Honoraires du notaire (% du prix client)</t>
+          <t>Taxes gouvernementales (% du prix client)</t>
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Honoraires du notaire - forfait minimum (IDR)</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="n">
-        <v>10000000</v>
+          <t>Honoraires du notaire (% du prix client)</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0.01</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Frais de geometre (EUR)</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="n">
-        <v>1000</v>
+          <t>Honoraires du notaire - forfait minimum (IDR)</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>10000000</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>Frais de geometre (EUR)</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>Taux d'acompte (appel de fonds)</t>
         </is>
       </c>
-      <c r="B17" s="5" t="n">
+      <c r="B18" s="5" t="n">
         <v>0.1</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>DETAIL DU CALCUL</t>
-        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
+          <t>DETAIL DU CALCUL</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
           <t>Poste</t>
         </is>
       </c>
-      <c r="B20" s="1" t="inlineStr">
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>Surface (ares)</t>
         </is>
       </c>
-      <c r="C20" s="1" t="inlineStr">
+      <c r="C21" s="1" t="inlineStr">
         <is>
           <t>Duree (ans)</t>
         </is>
       </c>
-      <c r="D20" s="1" t="inlineStr">
-        <is>
-          <t>Prix unitaire (IDR/are/an)</t>
-        </is>
-      </c>
-      <c r="E20" s="1" t="inlineStr">
+      <c r="D21" s="1" t="inlineStr">
+        <is>
+          <t>Prix unitaire (IDR / are / an)</t>
+        </is>
+      </c>
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>Montant IDR</t>
         </is>
       </c>
-      <c r="F20" s="1" t="inlineStr">
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>Montant EUR</t>
         </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Prix du terrain - PRIX VENDEUR</t>
-        </is>
-      </c>
-      <c r="B21" s="3">
-        <f>B7</f>
-        <v/>
-      </c>
-      <c r="C21" s="4">
-        <f>B9</f>
-        <v/>
-      </c>
-      <c r="D21" s="4">
-        <f>B10</f>
-        <v/>
-      </c>
-      <c r="E21" s="4">
-        <f>B21*C21*D21</f>
-        <v/>
-      </c>
-      <c r="F21" s="3">
-        <f>E21/$B$12</f>
-        <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Prix du terrain - PRIX CLIENT (avec commission)</t>
+          <t>Prix du terrain - PRIX VENDEUR</t>
         </is>
       </c>
       <c r="B22" s="3">
-        <f>B7</f>
+        <f>$B$8</f>
         <v/>
       </c>
       <c r="C22" s="4">
-        <f>B9</f>
+        <f>$B$10</f>
         <v/>
       </c>
       <c r="D22" s="4">
-        <f>B11</f>
+        <f>$B$11</f>
         <v/>
       </c>
       <c r="E22" s="4">
@@ -714,228 +694,262 @@
         <v/>
       </c>
       <c r="F22" s="3">
-        <f>E22/$B$12</f>
+        <f>E22/$B$13</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
+          <t>Prix du terrain - PRIX CLIENT (avec commission)</t>
+        </is>
+      </c>
+      <c r="B23" s="3">
+        <f>$B$8</f>
+        <v/>
+      </c>
+      <c r="C23" s="4">
+        <f>$B$10</f>
+        <v/>
+      </c>
+      <c r="D23" s="4">
+        <f>$B$12</f>
+        <v/>
+      </c>
+      <c r="E23" s="4">
+        <f>B23*C23*D23</f>
+        <v/>
+      </c>
+      <c r="F23" s="3">
+        <f>E23/$B$13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
           <t>dont commission agence (ecart vendeur / client)</t>
         </is>
       </c>
-      <c r="E23" s="4">
-        <f>E22-E21</f>
-        <v/>
-      </c>
-      <c r="F23" s="3">
-        <f>E23/$B$12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="1" t="inlineStr">
+      <c r="E24" s="4">
+        <f>E23-E22</f>
+        <v/>
+      </c>
+      <c r="F24" s="3">
+        <f>E24/$B$13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
         <is>
           <t>FRAIS ANNEXES</t>
         </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Taxes gouvernementales (5% du prix client)</t>
-        </is>
-      </c>
-      <c r="D26" s="5">
-        <f>B13</f>
-        <v/>
-      </c>
-      <c r="E26" s="4">
-        <f>E22*$B$13</f>
-        <v/>
-      </c>
-      <c r="F26" s="3">
-        <f>E26/$B$12</f>
-        <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Honoraires du notaire (1% du prix client, minimum 10 000 000 IDR)</t>
+          <t>Taxes gouvernementales (5% du prix client)</t>
         </is>
       </c>
       <c r="D27" s="5">
-        <f>IF(E22=0,0,E27/E22)</f>
+        <f>$B$14</f>
         <v/>
       </c>
       <c r="E27" s="4">
-        <f>MAX(E22*$B$14,$B$15)</f>
+        <f>E23*$B$14</f>
         <v/>
       </c>
       <c r="F27" s="3">
-        <f>E27/$B$12</f>
+        <f>E27/$B$13</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Sous-total frais de notaire (taxes + honoraires)</t>
+          <t>Honoraires du notaire (1% du prix client, minimum 10 000 000 IDR)</t>
         </is>
       </c>
       <c r="D28" s="5">
-        <f>IF(E22=0,0,E28/E22)</f>
+        <f>IF(E23=0,0,E28/E23)</f>
         <v/>
       </c>
       <c r="E28" s="4">
-        <f>E26+E27</f>
+        <f>MAX(E23*$B$15,$B$16)</f>
         <v/>
       </c>
       <c r="F28" s="3">
-        <f>E28/$B$12</f>
+        <f>E28/$B$13</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
+          <t>Sous-total frais de notaire (taxes + honoraires)</t>
+        </is>
+      </c>
+      <c r="D29" s="5">
+        <f>IF(E23=0,0,E29/E23)</f>
+        <v/>
+      </c>
+      <c r="E29" s="4">
+        <f>E27+E28</f>
+        <v/>
+      </c>
+      <c r="F29" s="3">
+        <f>E29/$B$13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
           <t>Frais de geometre (forfait 1 000 EUR)</t>
         </is>
       </c>
-      <c r="E29" s="4">
-        <f>$B$16*$B$12</f>
-        <v/>
-      </c>
-      <c r="F29" s="3">
-        <f>$B$16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="1" t="inlineStr">
+      <c r="E30" s="4">
+        <f>$B$17*$B$13</f>
+        <v/>
+      </c>
+      <c r="F30" s="3">
+        <f>$B$17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
         <is>
           <t>TOTAL DE L'OPERATION POUR L'ACHETEUR</t>
         </is>
       </c>
-      <c r="E31" s="6">
-        <f>E22+E28+E29</f>
-        <v/>
-      </c>
-      <c r="F31" s="7">
-        <f>E31/$B$12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="1" t="inlineStr">
+      <c r="E32" s="6">
+        <f>E23+E29+E30</f>
+        <v/>
+      </c>
+      <c r="F32" s="7">
+        <f>E32/$B$13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="inlineStr">
         <is>
           <t>APPEL DE FONDS</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="1" t="inlineStr">
         <is>
           <t>Acompte 10% du total de l'operation (reservation notaire)</t>
         </is>
       </c>
-      <c r="D34" s="5">
-        <f>B17</f>
-        <v/>
-      </c>
-      <c r="E34" s="6">
-        <f>E31*$B$17</f>
-        <v/>
-      </c>
-      <c r="F34" s="7">
-        <f>E34/$B$12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+      <c r="D35" s="5">
+        <f>$B$18</f>
+        <v/>
+      </c>
+      <c r="E35" s="6">
+        <f>E32*$B$18</f>
+        <v/>
+      </c>
+      <c r="F35" s="7">
+        <f>E35/$B$13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>Solde a regler apres acompte</t>
         </is>
       </c>
-      <c r="E35" s="4">
-        <f>E31-E34</f>
-        <v/>
-      </c>
-      <c r="F35" s="3">
-        <f>E35/$B$12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="E36" s="4">
+        <f>E32-E35</f>
+        <v/>
+      </c>
+      <c r="F36" s="3">
+        <f>E36/$B$13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>Pour information : 10% du prix du terrain seul</t>
         </is>
       </c>
-      <c r="E37" s="4">
-        <f>E22*$B$17</f>
-        <v/>
-      </c>
-      <c r="F37" s="3">
-        <f>E37/$B$12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="1" t="inlineStr">
+      <c r="E38" s="4">
+        <f>E23*$B$18</f>
+        <v/>
+      </c>
+      <c r="F38" s="3">
+        <f>E38/$B$13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="inlineStr">
         <is>
           <t>NOTES / HYPOTHESES</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>1 are = 100 m2 -&gt; terrain de 600 m2. Prix leasehold exprime en IDR par are et par an, sur 30 ans.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Taux de change en B12 : reference BCE du 20/08/2026 (1 EUR = 20 788,62 IDR). A actualiser avant envoi au client.</t>
+          <t>1 are = 100 m2 -&gt; terrain de 600 m2.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Frais de notaire detailles : taxes gouvernementales 5% (B13) + honoraires du notaire 1% (B14).</t>
+          <t>Achat en LEASEHOLD : prix exprime en IDR par are et par an, multiplie par la duree du bail.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Honoraires du notaire : le pourcentage s'applique sauf s'il donne moins que le forfait minimum de 10 000 000 IDR (B15), auquel cas le forfait est retenu (formule MAX en E27).</t>
+          <t>Taux de change en B13 : reference BCE du 20/08/2026 (1 EUR = 20 788,62 IDR). A actualiser avant envoi au client.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Ces taux sont appliques au prix client avec commission. Remplacer E22 par E21 dans les formules E26 et E27 si la base retenue est le prix vendeur.</t>
+          <t>Frais de notaire detailles : taxes gouvernementales 5% (B14) + honoraires du notaire 1% (B15).</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Frais de geometre saisis en EUR (B16) et convertis en IDR au taux B12.</t>
+          <t>Honoraires du notaire : le pourcentage s'applique sauf s'il donne moins que le forfait minimum de 10 000 000 IDR (B16), auquel cas le forfait est retenu (formule MAX en E28).</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Seules les cellules de parametres (colonne B, lignes 7 a 17) sont a saisir : tout le reste du tableau est calcule par formules et se met a jour automatiquement.</t>
+          <t>Ces taux sont appliques au prix client avec commission. Remplacer E23 par E22 dans les formules de frais si la base retenue est le prix vendeur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Frais de geometre saisis en EUR (B17) et convertis en IDR au taux B13.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Seules les cellules de parametres (colonne B, lignes 8 a 18) sont a saisir : tout le reste du tableau est calcule par formules et se met a jour automatiquement.</t>
         </is>
       </c>
     </row>

</xml_diff>